<commit_message>
New temporary leases law v0.1
</commit_message>
<xml_diff>
--- a/app/templates/report/recursos.xlsx
+++ b/app/templates/report/recursos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B20243D-06E7-4A95-89EC-F26F50C1211E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF632EB-7247-4457-902D-4E7D199B4117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">_Precios!$A$2:$N$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$AS$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$AT$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Valoraciones!$A$2:$F$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="123">
   <si>
     <t>Code</t>
   </si>
@@ -408,6 +408,12 @@
   </si>
   <si>
     <t>Rent_group</t>
+  </si>
+  <si>
+    <t>Superficie m2 sin comunes</t>
+  </si>
+  <si>
+    <t>Area_woc</t>
   </si>
 </sst>
 </file>
@@ -995,7 +1001,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AT3"/>
+  <dimension ref="A1:AU3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="37.28515625" style="2" customWidth="1"/>
@@ -1019,17 +1025,17 @@
     <col min="29" max="30" width="11.85546875" style="2" customWidth="1"/>
     <col min="31" max="33" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="34" max="35" width="15.42578125" style="2" customWidth="1"/>
-    <col min="36" max="36" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="12.7109375" style="2" customWidth="1"/>
-    <col min="39" max="40" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="41" max="44" width="16.85546875" style="2" customWidth="1"/>
-    <col min="45" max="45" width="20.5703125" style="2" customWidth="1"/>
-    <col min="46" max="46" width="5" style="2" bestFit="1" customWidth="1"/>
-    <col min="47" max="16384" width="24.85546875" style="2"/>
+    <col min="36" max="37" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="12.7109375" style="2" customWidth="1"/>
+    <col min="40" max="41" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="42" max="45" width="16.85546875" style="2" customWidth="1"/>
+    <col min="46" max="46" width="20.5703125" style="2" customWidth="1"/>
+    <col min="47" max="47" width="5" style="2" bestFit="1" customWidth="1"/>
+    <col min="48" max="16384" width="24.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:47" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1135,38 +1141,41 @@
         <v>15</v>
       </c>
       <c r="AK1" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="AL1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="AL1" s="3" t="s">
+      <c r="AM1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AN1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="AN1" s="3" t="s">
+      <c r="AO1" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="AO1" s="3" t="s">
+      <c r="AP1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AP1" s="3" t="s">
+      <c r="AQ1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AQ1" s="3" t="s">
+      <c r="AR1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="AR1" s="3" t="s">
+      <c r="AS1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AS1" s="3" t="s">
+      <c r="AT1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AT1" s="1">
+      <c r="AU1" s="1">
         <f ca="1">IF(MONTH(TODAY())&gt;8,1+YEAR(TODAY()),YEAR(TODAY()))</f>
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>67</v>
       </c>
@@ -1258,34 +1267,37 @@
         <v>14</v>
       </c>
       <c r="AK2" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="AL2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="AL2" s="4" t="s">
+      <c r="AM2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="AM2" s="4" t="s">
+      <c r="AN2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="AN2" s="4" t="s">
+      <c r="AO2" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="AO2" s="4" t="s">
+      <c r="AP2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="AP2" s="4" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AS2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="10"/>
@@ -1303,23 +1315,23 @@
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
       <c r="Q3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AT$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="R3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AT$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="S3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AT$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="T3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AT$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
         <v>0</v>
       </c>
       <c r="U3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AT$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
         <v>0</v>
       </c>
       <c r="V3" s="13">
@@ -1357,10 +1369,11 @@
       <c r="AQ3" s="10"/>
       <c r="AR3" s="10"/>
       <c r="AS3" s="10"/>
+      <c r="AT3" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AS3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A3:AS9991">
+  <autoFilter ref="A2:AT3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A3:AT9991">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>LEN($D3)=12</formula>
     </cfRule>
@@ -1834,6 +1847,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="220d4249-f262-4642-a86b-ff46de6e315d">
@@ -1842,15 +1864,6 @@
     <TaxCatchAll xmlns="965e701d-44ad-4371-a199-8fefe953808c"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1873,6 +1886,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC650EC1-3E41-4FC6-BA6C-52921951A8DA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1881,12 +1902,4 @@
     <ds:schemaRef ds:uri="965e701d-44ad-4371-a199-8fefe953808c"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Resources export w/new mgmt fee
</commit_message>
<xml_diff>
--- a/app/templates/report/recursos.xlsx
+++ b/app/templates/report/recursos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF632EB-7247-4457-902D-4E7D199B4117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFDE5250-B370-4E74-BFA1-8CB23631D3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">_Precios!$A$2:$N$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$AT$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$AX$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Valoraciones!$A$2:$F$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="131">
   <si>
     <t>Code</t>
   </si>
@@ -299,9 +299,6 @@
     <t>Management_fee</t>
   </si>
   <si>
-    <t>Management fee</t>
-  </si>
-  <si>
     <t>Uso</t>
   </si>
   <si>
@@ -414,6 +411,38 @@
   </si>
   <si>
     <t>Area_woc</t>
+  </si>
+  <si>
+    <t>M. Fee
+Sin servicios</t>
+  </si>
+  <si>
+    <t>M. Fee
+Semanal</t>
+  </si>
+  <si>
+    <t>M. Fee
+No limpieza</t>
+  </si>
+  <si>
+    <t>M. Fee
+Quincenal</t>
+  </si>
+  <si>
+    <t>M. Fee
+Mensual</t>
+  </si>
+  <si>
+    <t>Management_fee_no_cleaning</t>
+  </si>
+  <si>
+    <t>Management_fee_weekly</t>
+  </si>
+  <si>
+    <t>Management_fee_biweekly</t>
+  </si>
+  <si>
+    <t>Management_fee_monthly</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +1030,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AU3"/>
+  <dimension ref="A1:AY3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="37.28515625" style="2" customWidth="1"/>
@@ -1016,26 +1045,26 @@
     <col min="13" max="13" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="24" width="9.5703125" style="2" customWidth="1"/>
-    <col min="25" max="25" width="30" style="2" customWidth="1"/>
-    <col min="26" max="26" width="10.7109375" style="2" customWidth="1"/>
-    <col min="27" max="27" width="30" style="2" customWidth="1"/>
-    <col min="28" max="28" width="24.7109375" style="2" customWidth="1"/>
-    <col min="29" max="30" width="11.85546875" style="2" customWidth="1"/>
-    <col min="31" max="33" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="15.42578125" style="2" customWidth="1"/>
-    <col min="36" max="37" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="12.7109375" style="2" customWidth="1"/>
-    <col min="40" max="41" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="42" max="45" width="16.85546875" style="2" customWidth="1"/>
-    <col min="46" max="46" width="20.5703125" style="2" customWidth="1"/>
-    <col min="47" max="47" width="5" style="2" bestFit="1" customWidth="1"/>
-    <col min="48" max="16384" width="24.85546875" style="2"/>
+    <col min="16" max="20" width="12.28515625" style="2" customWidth="1"/>
+    <col min="21" max="28" width="9.5703125" style="2" customWidth="1"/>
+    <col min="29" max="29" width="30" style="2" customWidth="1"/>
+    <col min="30" max="30" width="10.7109375" style="2" customWidth="1"/>
+    <col min="31" max="31" width="30" style="2" customWidth="1"/>
+    <col min="32" max="32" width="24.7109375" style="2" customWidth="1"/>
+    <col min="33" max="34" width="11.85546875" style="2" customWidth="1"/>
+    <col min="35" max="37" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="38" max="39" width="15.42578125" style="2" customWidth="1"/>
+    <col min="40" max="41" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="12.7109375" style="2" customWidth="1"/>
+    <col min="44" max="45" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="46" max="49" width="16.85546875" style="2" customWidth="1"/>
+    <col min="50" max="50" width="20.5703125" style="2" customWidth="1"/>
+    <col min="51" max="51" width="5" style="2" bestFit="1" customWidth="1"/>
+    <col min="52" max="16384" width="24.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:51" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1043,7 +1072,7 @@
         <v>68</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>33</v>
@@ -1078,104 +1107,116 @@
         <v>5</v>
       </c>
       <c r="P1" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="AD1" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="AE1" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="AF1" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="Q1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="Z1" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="AB1" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="AD1" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AI1" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="AJ1" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AK1" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="AG1" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="AH1" s="3" t="s">
+      <c r="AL1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="AI1" s="3" t="s">
+      <c r="AM1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="AJ1" s="3" t="s">
+      <c r="AN1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="AK1" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="AL1" s="3" t="s">
+      <c r="AO1" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="AP1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AQ1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AN1" s="3" t="s">
+      <c r="AR1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="AO1" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AP1" s="3" t="s">
+      <c r="AS1" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AQ1" s="3" t="s">
+      <c r="AU1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AR1" s="3" t="s">
+      <c r="AV1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="AS1" s="3" t="s">
+      <c r="AW1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AT1" s="3" t="s">
+      <c r="AX1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AU1" s="1">
+      <c r="AY1" s="1">
         <f ca="1">IF(MONTH(TODAY())&gt;8,1+YEAR(TODAY()),YEAR(TODAY()))</f>
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>67</v>
       </c>
@@ -1183,7 +1224,7 @@
         <v>69</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>0</v>
@@ -1222,82 +1263,94 @@
       <c r="P2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
+      <c r="Q2" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>130</v>
+      </c>
       <c r="U2" s="4"/>
       <c r="V2" s="4"/>
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
-      <c r="Y2" s="4" t="s">
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
+      <c r="AA2" s="4"/>
+      <c r="AB2" s="4"/>
+      <c r="AC2" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="AD2" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="Z2" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="AA2" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="AB2" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="AC2" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="AD2" s="4" t="s">
-        <v>103</v>
-      </c>
       <c r="AE2" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="AF2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="AG2" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="AH2" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="AI2" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="AJ2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="AF2" s="4" t="s">
+      <c r="AK2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="AG2" s="4" t="s">
+      <c r="AL2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="AM2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="AN2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="AO2" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="AP2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AR2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AS2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="AH2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="AI2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="AJ2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="AK2" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="AL2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="AM2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="AN2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="AO2" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="AP2" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AV2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AW2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AX2" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="10"/>
@@ -1314,50 +1367,50 @@
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
-      <c r="Q3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($AY$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
-      <c r="R3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+      <c r="V3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($AY$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
-      <c r="S3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+      <c r="W3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($AY$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
-      <c r="T3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
+      <c r="X3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($AY$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
         <v>0</v>
       </c>
-      <c r="U3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($AU$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
+      <c r="Y3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($AY$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
         <v>0</v>
       </c>
-      <c r="V3" s="13">
-        <f t="shared" ref="V3" ca="1" si="0">$Q3+$U3</f>
+      <c r="Z3" s="13">
+        <f t="shared" ref="Z3" ca="1" si="0">$U3+$Y3</f>
         <v>0</v>
       </c>
-      <c r="W3" s="13">
-        <f t="shared" ref="W3" ca="1" si="1">$R3+$U3</f>
+      <c r="AA3" s="13">
+        <f t="shared" ref="AA3" ca="1" si="1">$V3+$Y3</f>
         <v>0</v>
       </c>
-      <c r="X3" s="13">
-        <f t="shared" ref="X3" ca="1" si="2">$S3+$U3</f>
+      <c r="AB3" s="13">
+        <f t="shared" ref="AB3" ca="1" si="2">$W3+$Y3</f>
         <v>0</v>
       </c>
-      <c r="Y3" s="21"/>
-      <c r="Z3" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="AA3" s="21"/>
-      <c r="AB3" s="17"/>
-      <c r="AC3" s="18"/>
-      <c r="AD3" s="20"/>
-      <c r="AE3" s="10"/>
-      <c r="AF3" s="10"/>
-      <c r="AG3" s="10"/>
-      <c r="AH3" s="10"/>
+      <c r="AC3" s="21"/>
+      <c r="AD3" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="AE3" s="21"/>
+      <c r="AF3" s="17"/>
+      <c r="AG3" s="18"/>
+      <c r="AH3" s="20"/>
       <c r="AI3" s="10"/>
       <c r="AJ3" s="10"/>
       <c r="AK3" s="10"/>
@@ -1370,10 +1423,14 @@
       <c r="AR3" s="10"/>
       <c r="AS3" s="10"/>
       <c r="AT3" s="10"/>
+      <c r="AU3" s="10"/>
+      <c r="AV3" s="10"/>
+      <c r="AW3" s="10"/>
+      <c r="AX3" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AT3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A3:AT9991">
+  <autoFilter ref="A2:AX3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A3:AX9991">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>LEN($D3)=12</formula>
     </cfRule>
@@ -1400,45 +1457,45 @@
         <v>33</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>112</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E2" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="10"/>
       <c r="B3" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C3" s="18"/>
       <c r="D3" s="18"/>
@@ -1500,7 +1557,7 @@
         <v>41</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>42</v>
@@ -1550,7 +1607,7 @@
         <v>51</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L2" s="4" t="s">
         <v>52</v>
@@ -1847,15 +1904,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="220d4249-f262-4642-a86b-ff46de6e315d">
@@ -1864,6 +1912,15 @@
     <TaxCatchAll xmlns="965e701d-44ad-4371-a199-8fefe953808c"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1886,14 +1943,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC650EC1-3E41-4FC6-BA6C-52921951A8DA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1902,4 +1951,12 @@
     <ds:schemaRef ds:uri="965e701d-44ad-4371-a199-8fefe953808c"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Calc LAW prices v0.2
</commit_message>
<xml_diff>
--- a/app/templates/report/recursos.xlsx
+++ b/app/templates/report/recursos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7317523B-AB4F-4B3F-84D9-8C6070D85C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C4C6AB-E32B-4C6E-B088-360BD108F574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Recursos" sheetId="37" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">_Precios!$A$2:$N$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BH$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BJ$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Valoraciones!$A$2:$F$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="154">
   <si>
     <t>Code</t>
   </si>
@@ -501,6 +501,18 @@
   </si>
   <si>
     <t>Occupancy_certificate</t>
+  </si>
+  <si>
+    <t>Consumos</t>
+  </si>
+  <si>
+    <t>Max_utility</t>
+  </si>
+  <si>
+    <t>Repercutir Gastos Comunidad</t>
+  </si>
+  <si>
+    <t>HOA</t>
   </si>
 </sst>
 </file>
@@ -651,7 +663,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -703,6 +715,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="3" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1114,46 +1135,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BI3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BK3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="37.28515625" style="2" customWidth="1"/>
-    <col min="3" max="4" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="20.42578125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="29.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.85546875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="20" width="12.28515625" style="2" customWidth="1"/>
-    <col min="21" max="28" width="9.5703125" style="2" customWidth="1"/>
+    <col min="1" max="2" width="37.33203125" style="2" customWidth="1"/>
+    <col min="3" max="4" width="20.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="20.44140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.88671875" style="2" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="20" width="12.33203125" style="2" customWidth="1"/>
+    <col min="21" max="28" width="9.5546875" style="2" customWidth="1"/>
     <col min="29" max="29" width="30" style="2" customWidth="1"/>
-    <col min="30" max="30" width="10.7109375" style="2" customWidth="1"/>
+    <col min="30" max="30" width="10.6640625" style="2" customWidth="1"/>
     <col min="31" max="31" width="30" style="2" customWidth="1"/>
-    <col min="32" max="32" width="24.7109375" style="2" customWidth="1"/>
-    <col min="33" max="33" width="11.85546875" style="2" customWidth="1"/>
-    <col min="34" max="35" width="10.7109375" style="2" customWidth="1"/>
-    <col min="36" max="37" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="10.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="39" max="43" width="10.7109375" style="2" customWidth="1"/>
-    <col min="44" max="44" width="11.85546875" style="2" customWidth="1"/>
-    <col min="45" max="47" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="48" max="49" width="15.42578125" style="2" customWidth="1"/>
-    <col min="50" max="51" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="12.7109375" style="2" customWidth="1"/>
-    <col min="54" max="55" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="56" max="59" width="16.85546875" style="2" customWidth="1"/>
-    <col min="60" max="60" width="20.5703125" style="2" customWidth="1"/>
-    <col min="61" max="61" width="5.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="62" max="16384" width="24.85546875" style="2"/>
+    <col min="32" max="32" width="24.6640625" style="2" customWidth="1"/>
+    <col min="33" max="33" width="11.88671875" style="2" customWidth="1"/>
+    <col min="34" max="35" width="10.6640625" style="2" customWidth="1"/>
+    <col min="36" max="37" width="17.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="10.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="39" max="44" width="10.6640625" style="2" customWidth="1"/>
+    <col min="45" max="45" width="14.109375" style="28" customWidth="1"/>
+    <col min="46" max="46" width="11.88671875" style="2" customWidth="1"/>
+    <col min="47" max="49" width="17.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="50" max="51" width="15.44140625" style="2" customWidth="1"/>
+    <col min="52" max="53" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="12.6640625" style="2" customWidth="1"/>
+    <col min="56" max="57" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="58" max="61" width="16.88671875" style="2" customWidth="1"/>
+    <col min="62" max="62" width="20.5546875" style="2" customWidth="1"/>
+    <col min="63" max="63" width="5.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="64" max="16384" width="24.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:61" s="1" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:63" s="1" customFormat="1" ht="37.799999999999997" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1277,65 +1299,71 @@
         <v>42</v>
       </c>
       <c r="AQ1" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="AR1" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="AR1" s="3" t="s">
+      <c r="AS1" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="AT1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="AS1" s="3" t="s">
+      <c r="AU1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="AT1" s="3" t="s">
+      <c r="AV1" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AU1" s="3" t="s">
+      <c r="AW1" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="AV1" s="3" t="s">
+      <c r="AX1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="AW1" s="3" t="s">
+      <c r="AY1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="AX1" s="3" t="s">
+      <c r="AZ1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="AY1" s="3" t="s">
+      <c r="BA1" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="AZ1" s="3" t="s">
+      <c r="BB1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="BA1" s="3" t="s">
+      <c r="BC1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BD1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BE1" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BF1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BG1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="BF1" s="3" t="s">
+      <c r="BH1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="BG1" s="3" t="s">
+      <c r="BI1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="BH1" s="3" t="s">
+      <c r="BJ1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="BI1" s="1">
+      <c r="BK1" s="1">
         <f ca="1">IF(MONTH(TODAY())&gt;8,1+YEAR(TODAY()),YEAR(TODAY()))</f>
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>67</v>
       </c>
@@ -1445,61 +1473,67 @@
         <v>146</v>
       </c>
       <c r="AQ2" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="AR2" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AS2" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="AT2" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AV2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="AU2" s="4" t="s">
+      <c r="AW2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="AV2" s="4" t="s">
+      <c r="AX2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="AW2" s="4" t="s">
+      <c r="AY2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="AX2" s="4" t="s">
+      <c r="AZ2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="AY2" s="4" t="s">
+      <c r="BA2" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="AZ2" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="BA2" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="BB2" s="4" t="s">
+      <c r="BD2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="BC2" s="4" t="s">
+      <c r="BE2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="BD2" s="4" t="s">
+      <c r="BF2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="BE2" s="4" t="s">
+      <c r="BG2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="BF2" s="4" t="s">
+      <c r="BH2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="BG2" s="4" t="s">
+      <c r="BI2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="BH2" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="10"/>
@@ -1521,23 +1555,23 @@
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BI$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="V3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BI$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="W3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BI$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="X3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BI$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
         <v>0</v>
       </c>
       <c r="Y3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BI$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
         <v>0</v>
       </c>
       <c r="Z3" s="13">
@@ -1575,9 +1609,9 @@
       <c r="AO3" s="24"/>
       <c r="AP3" s="24"/>
       <c r="AQ3" s="24"/>
-      <c r="AR3" s="18"/>
-      <c r="AS3" s="10"/>
-      <c r="AT3" s="10"/>
+      <c r="AR3" s="24"/>
+      <c r="AS3" s="27"/>
+      <c r="AT3" s="18"/>
       <c r="AU3" s="10"/>
       <c r="AV3" s="10"/>
       <c r="AW3" s="10"/>
@@ -1592,10 +1626,12 @@
       <c r="BF3" s="10"/>
       <c r="BG3" s="10"/>
       <c r="BH3" s="10"/>
+      <c r="BI3" s="10"/>
+      <c r="BJ3" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BH3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A3:BH9990">
+  <autoFilter ref="A2:BJ3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A3:BJ9990">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>LEN($D3)=12</formula>
     </cfRule>
@@ -1609,12 +1645,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E1D64B2-929E-46C9-92E4-4B6A6392A32E}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" style="2" customWidth="1"/>
     <col min="3" max="6" width="14" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="24.85546875" style="2"/>
+    <col min="7" max="16384" width="24.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1683,17 +1719,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F063E8C-9C12-4A86-8416-6A77642A363A}">
   <dimension ref="A1:S3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="40.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="18" width="17.7109375" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="24.85546875" style="2"/>
+    <col min="1" max="1" width="9.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="40.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="18" width="17.6640625" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="24.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1830,12 +1866,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F48469C1-5DA9-43F7-A0B7-76DC91FAD532}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="7.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Calc LAW prices v0.6 fixes
</commit_message>
<xml_diff>
--- a/app/templates/report/recursos.xlsx
+++ b/app/templates/report/recursos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72E2178-D727-436A-A1D9-C108A6D97E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019FB0BB-8B03-4545-94B2-5CA1203490E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -509,10 +509,10 @@
     <t>Max_utility</t>
   </si>
   <si>
-    <t>Repercutir Gastos Comunidad</t>
-  </si>
-  <si>
     <t>HOA</t>
+  </si>
+  <si>
+    <t>Repercutir Gastos</t>
   </si>
 </sst>
 </file>
@@ -1180,7 +1180,7 @@
     <col min="64" max="16384" width="24.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:63" s="1" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:63" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>138</v>
       </c>
       <c r="AS1" s="21" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AT1" s="3" t="s">
         <v>99</v>
@@ -1484,7 +1484,7 @@
         <v>147</v>
       </c>
       <c r="AS2" s="25" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AT2" s="4" t="s">
         <v>100</v>
@@ -2110,15 +2110,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="220d4249-f262-4642-a86b-ff46de6e315d">
@@ -2127,6 +2118,15 @@
     <TaxCatchAll xmlns="965e701d-44ad-4371-a199-8fefe953808c"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2149,14 +2149,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC650EC1-3E41-4FC6-BA6C-52921951A8DA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2165,4 +2157,12 @@
     <ds:schemaRef ds:uri="965e701d-44ad-4371-a199-8fefe953808c"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix LAW calculation and report
</commit_message>
<xml_diff>
--- a/app/templates/report/recursos.xlsx
+++ b/app/templates/report/recursos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019FB0BB-8B03-4545-94B2-5CA1203490E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BE9E5A-197C-4F26-B03E-F78217B6B69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">_Precios!$A$2:$N$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BJ$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BN$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Valoraciones!$A$2:$F$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="158">
   <si>
     <t>Code</t>
   </si>
@@ -513,6 +513,18 @@
   </si>
   <si>
     <t>Repercutir Gastos</t>
+  </si>
+  <si>
+    <t>Tipo de afectación</t>
+  </si>
+  <si>
+    <t>Renta máxima LAU</t>
+  </si>
+  <si>
+    <t>Renta máxima</t>
+  </si>
+  <si>
+    <t>Gastos repecut.</t>
   </si>
 </sst>
 </file>
@@ -572,7 +584,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -612,6 +624,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF009E93"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -662,7 +686,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -729,6 +753,11 @@
     <xf numFmtId="2" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -827,6 +856,7 @@
       <rgbColor rgb="00333333"/>
     </indexedColors>
     <mruColors>
+      <color rgb="FF009E93"/>
       <color rgb="FF008A80"/>
       <color rgb="FFD1FFFC"/>
     </mruColors>
@@ -1139,7 +1169,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BK3"/>
+  <dimension ref="A1:BO3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="37.28515625" style="2" customWidth="1"/>
@@ -1167,20 +1197,20 @@
     <col min="39" max="39" width="11.5703125" style="2" customWidth="1"/>
     <col min="40" max="44" width="10.7109375" style="2" customWidth="1"/>
     <col min="45" max="45" width="14.140625" style="27" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" style="2" customWidth="1"/>
-    <col min="47" max="49" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="50" max="51" width="15.42578125" style="2" customWidth="1"/>
-    <col min="52" max="53" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="12.7109375" style="2" customWidth="1"/>
-    <col min="56" max="57" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="58" max="61" width="16.85546875" style="2" customWidth="1"/>
-    <col min="62" max="62" width="20.5703125" style="2" customWidth="1"/>
-    <col min="63" max="63" width="5.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="64" max="16384" width="24.85546875" style="2"/>
+    <col min="46" max="50" width="11.85546875" style="2" customWidth="1"/>
+    <col min="51" max="53" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="54" max="55" width="15.42578125" style="2" customWidth="1"/>
+    <col min="56" max="57" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="12.7109375" style="2" customWidth="1"/>
+    <col min="60" max="61" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="62" max="65" width="16.85546875" style="2" customWidth="1"/>
+    <col min="66" max="66" width="20.5703125" style="2" customWidth="1"/>
+    <col min="67" max="67" width="5.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="68" max="16384" width="24.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:63" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:67" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1312,63 +1342,75 @@
       <c r="AS1" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="AT1" s="3" t="s">
+      <c r="AT1" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="AU1" s="32" t="s">
+        <v>155</v>
+      </c>
+      <c r="AV1" s="32" t="s">
+        <v>156</v>
+      </c>
+      <c r="AW1" s="32" t="s">
+        <v>157</v>
+      </c>
+      <c r="AX1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="AU1" s="3" t="s">
+      <c r="AY1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="AV1" s="3" t="s">
+      <c r="AZ1" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AW1" s="3" t="s">
+      <c r="BA1" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="AX1" s="3" t="s">
+      <c r="BB1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="AY1" s="3" t="s">
+      <c r="BC1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="AZ1" s="3" t="s">
+      <c r="BD1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="BA1" s="3" t="s">
+      <c r="BE1" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BF1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BG1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BH1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BI1" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="BF1" s="3" t="s">
+      <c r="BJ1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="BG1" s="3" t="s">
+      <c r="BK1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="BH1" s="3" t="s">
+      <c r="BL1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="BI1" s="3" t="s">
+      <c r="BM1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="BJ1" s="3" t="s">
+      <c r="BN1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="BK1" s="1">
+      <c r="BO1" s="1">
         <f ca="1">IF(MONTH(TODAY())&gt;8,1+YEAR(TODAY()),YEAR(TODAY()))</f>
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:63" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>67</v>
       </c>
@@ -1486,59 +1528,63 @@
       <c r="AS2" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AT2" s="4"/>
+      <c r="AU2" s="4"/>
+      <c r="AV2" s="4"/>
+      <c r="AW2" s="4"/>
+      <c r="AX2" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="AU2" s="4" t="s">
+      <c r="AY2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="AV2" s="4" t="s">
+      <c r="AZ2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="AW2" s="4" t="s">
+      <c r="BA2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="AX2" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="AY2" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="AZ2" s="4" t="s">
+      <c r="BD2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="BA2" s="4" t="s">
+      <c r="BE2" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="BB2" s="4" t="s">
+      <c r="BF2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="BC2" s="4" t="s">
+      <c r="BG2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="BD2" s="4" t="s">
+      <c r="BH2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="BE2" s="4" t="s">
+      <c r="BI2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="BF2" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="BG2" s="4" t="s">
+      <c r="BK2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="BH2" s="4" t="s">
+      <c r="BL2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="BI2" s="4" t="s">
+      <c r="BM2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="BJ2" s="4" t="s">
+      <c r="BN2" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:63" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:67" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="10"/>
@@ -1560,23 +1606,23 @@
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="V3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="W3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="X3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
         <v>0</v>
       </c>
       <c r="Y3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BK$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
         <v>0</v>
       </c>
       <c r="Z3" s="13">
@@ -1616,11 +1662,11 @@
       <c r="AQ3" s="23"/>
       <c r="AR3" s="23"/>
       <c r="AS3" s="26"/>
-      <c r="AT3" s="18"/>
-      <c r="AU3" s="10"/>
-      <c r="AV3" s="10"/>
-      <c r="AW3" s="10"/>
-      <c r="AX3" s="10"/>
+      <c r="AT3" s="33"/>
+      <c r="AU3" s="34"/>
+      <c r="AV3" s="34"/>
+      <c r="AW3" s="34"/>
+      <c r="AX3" s="18"/>
       <c r="AY3" s="10"/>
       <c r="AZ3" s="10"/>
       <c r="BA3" s="10"/>
@@ -1633,10 +1679,14 @@
       <c r="BH3" s="10"/>
       <c r="BI3" s="10"/>
       <c r="BJ3" s="10"/>
+      <c r="BK3" s="10"/>
+      <c r="BL3" s="10"/>
+      <c r="BM3" s="10"/>
+      <c r="BN3" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BJ3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A3:BJ9988">
+  <autoFilter ref="A2:BN3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A3:BN9988">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>LEN($D3)=12</formula>
     </cfRule>
@@ -1913,6 +1963,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="220d4249-f262-4642-a86b-ff46de6e315d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="965e701d-44ad-4371-a199-8fefe953808c"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001BDC921D6C313740BA67D7760DC75571" ma:contentTypeVersion="9" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ec6cd274e87ab0abf30bec2e834aaf15">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="220d4249-f262-4642-a86b-ff46de6e315d" xmlns:ns3="965e701d-44ad-4371-a199-8fefe953808c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e77808c4f084d99d477d3de919e85b9" ns2:_="" ns3:_="">
     <xsd:import namespace="220d4249-f262-4642-a86b-ff46de6e315d"/>
@@ -2109,27 +2179,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="220d4249-f262-4642-a86b-ff46de6e315d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="965e701d-44ad-4371-a199-8fefe953808c"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC650EC1-3E41-4FC6-BA6C-52921951A8DA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="220d4249-f262-4642-a86b-ff46de6e315d"/>
+    <ds:schemaRef ds:uri="965e701d-44ad-4371-a199-8fefe953808c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2190EF49-E186-4D77-87E3-BC317999ED9E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2146,23 +2215,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC650EC1-3E41-4FC6-BA6C-52921951A8DA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="220d4249-f262-4642-a86b-ff46de6e315d"/>
-    <ds:schemaRef ds:uri="965e701d-44ad-4371-a199-8fefe953808c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
New field in resources
</commit_message>
<xml_diff>
--- a/app/templates/report/recursos.xlsx
+++ b/app/templates/report/recursos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BE9E5A-197C-4F26-B03E-F78217B6B69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB8E3A73-690F-4BBF-A92D-4C5652B362CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">_Precios!$A$2:$N$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BN$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BO$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Valoraciones!$A$2:$F$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="160">
   <si>
     <t>Code</t>
   </si>
@@ -512,9 +512,6 @@
     <t>HOA</t>
   </si>
   <si>
-    <t>Repercutir Gastos</t>
-  </si>
-  <si>
     <t>Tipo de afectación</t>
   </si>
   <si>
@@ -525,6 +522,15 @@
   </si>
   <si>
     <t>Gastos repecut.</t>
+  </si>
+  <si>
+    <t>LAU aplicable?</t>
+  </si>
+  <si>
+    <t>Repercutir Gastos?</t>
+  </si>
+  <si>
+    <t>LAU_applicable</t>
   </si>
 </sst>
 </file>
@@ -1169,7 +1175,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BO3"/>
+  <dimension ref="A1:BP3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="37.28515625" style="2" customWidth="1"/>
@@ -1195,22 +1201,24 @@
     <col min="36" max="37" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="10.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="11.5703125" style="2" customWidth="1"/>
-    <col min="40" max="44" width="10.7109375" style="2" customWidth="1"/>
-    <col min="45" max="45" width="14.140625" style="27" customWidth="1"/>
-    <col min="46" max="50" width="11.85546875" style="2" customWidth="1"/>
-    <col min="51" max="53" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="54" max="55" width="15.42578125" style="2" customWidth="1"/>
-    <col min="56" max="57" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="12.7109375" style="2" customWidth="1"/>
-    <col min="60" max="61" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="62" max="65" width="16.85546875" style="2" customWidth="1"/>
-    <col min="66" max="66" width="20.5703125" style="2" customWidth="1"/>
-    <col min="67" max="67" width="5.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="68" max="16384" width="24.85546875" style="2"/>
+    <col min="40" max="40" width="10.7109375" style="2" customWidth="1"/>
+    <col min="41" max="41" width="14.140625" style="27" customWidth="1"/>
+    <col min="42" max="45" width="10.7109375" style="2" customWidth="1"/>
+    <col min="46" max="46" width="14.140625" style="27" customWidth="1"/>
+    <col min="47" max="51" width="11.85546875" style="2" customWidth="1"/>
+    <col min="52" max="54" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="55" max="56" width="15.42578125" style="2" customWidth="1"/>
+    <col min="57" max="58" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.7109375" style="2" customWidth="1"/>
+    <col min="61" max="62" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="63" max="66" width="16.85546875" style="2" customWidth="1"/>
+    <col min="67" max="67" width="20.5703125" style="2" customWidth="1"/>
+    <col min="68" max="68" width="5.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="69" max="16384" width="24.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:67" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:68" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1328,89 +1336,92 @@
         <v>136</v>
       </c>
       <c r="AO1" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="AP1" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="AP1" s="21" t="s">
+      <c r="AQ1" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="AQ1" s="21" t="s">
+      <c r="AR1" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="AR1" s="21" t="s">
+      <c r="AS1" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="AS1" s="21" t="s">
+      <c r="AT1" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="AU1" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="AT1" s="32" t="s">
+      <c r="AV1" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="AU1" s="32" t="s">
+      <c r="AW1" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="AV1" s="32" t="s">
+      <c r="AX1" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="AW1" s="32" t="s">
-        <v>157</v>
-      </c>
-      <c r="AX1" s="3" t="s">
+      <c r="AY1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="AY1" s="3" t="s">
+      <c r="AZ1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="AZ1" s="3" t="s">
+      <c r="BA1" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="BA1" s="3" t="s">
+      <c r="BB1" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BC1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BD1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BE1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BF1" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="BF1" s="3" t="s">
+      <c r="BG1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="BG1" s="3" t="s">
+      <c r="BH1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="BH1" s="3" t="s">
+      <c r="BI1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="BI1" s="3" t="s">
+      <c r="BJ1" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="BJ1" s="3" t="s">
+      <c r="BK1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="BK1" s="3" t="s">
+      <c r="BL1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="BL1" s="3" t="s">
+      <c r="BM1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="BM1" s="3" t="s">
+      <c r="BN1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="BN1" s="3" t="s">
+      <c r="BO1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="BO1" s="1">
+      <c r="BP1" s="1">
         <f ca="1">IF(MONTH(TODAY())&gt;8,1+YEAR(TODAY()),YEAR(TODAY()))</f>
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>67</v>
       </c>
@@ -1513,78 +1524,81 @@
       <c r="AN2" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="AO2" s="4" t="s">
+      <c r="AO2" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="AP2" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="AP2" s="4" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AS2" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="AS2" s="25" t="s">
+      <c r="AT2" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="AT2" s="4"/>
       <c r="AU2" s="4"/>
       <c r="AV2" s="4"/>
       <c r="AW2" s="4"/>
-      <c r="AX2" s="4" t="s">
+      <c r="AX2" s="4"/>
+      <c r="AY2" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="AY2" s="4" t="s">
+      <c r="AZ2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="AZ2" s="4" t="s">
+      <c r="BA2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="BA2" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="BB2" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="BC2" s="4" t="s">
+      <c r="BD2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="BD2" s="4" t="s">
+      <c r="BE2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="BE2" s="4" t="s">
+      <c r="BF2" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="BF2" s="4" t="s">
+      <c r="BG2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="BG2" s="4" t="s">
+      <c r="BH2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="BH2" s="4" t="s">
+      <c r="BI2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="BI2" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="BJ2" s="4" t="s">
+      <c r="BK2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="BK2" s="4" t="s">
+      <c r="BL2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="BL2" s="4" t="s">
+      <c r="BM2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="BM2" s="4" t="s">
+      <c r="BN2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="BN2" s="4" t="s">
+      <c r="BO2" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="10"/>
@@ -1606,23 +1620,23 @@
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="V3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="W3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="X3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
         <v>0</v>
       </c>
       <c r="Y3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BO$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
         <v>0</v>
       </c>
       <c r="Z3" s="13">
@@ -1657,17 +1671,17 @@
         <v>96</v>
       </c>
       <c r="AN3" s="23"/>
-      <c r="AO3" s="23"/>
+      <c r="AO3" s="26"/>
       <c r="AP3" s="23"/>
       <c r="AQ3" s="23"/>
       <c r="AR3" s="23"/>
-      <c r="AS3" s="26"/>
-      <c r="AT3" s="33"/>
-      <c r="AU3" s="34"/>
+      <c r="AS3" s="23"/>
+      <c r="AT3" s="26"/>
+      <c r="AU3" s="33"/>
       <c r="AV3" s="34"/>
       <c r="AW3" s="34"/>
-      <c r="AX3" s="18"/>
-      <c r="AY3" s="10"/>
+      <c r="AX3" s="34"/>
+      <c r="AY3" s="18"/>
       <c r="AZ3" s="10"/>
       <c r="BA3" s="10"/>
       <c r="BB3" s="10"/>
@@ -1683,10 +1697,11 @@
       <c r="BL3" s="10"/>
       <c r="BM3" s="10"/>
       <c r="BN3" s="10"/>
+      <c r="BO3" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BN3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A3:BN9988">
+  <autoFilter ref="A2:BO3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A3:BO9988">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>LEN($D3)=12</formula>
     </cfRule>
@@ -1974,15 +1989,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001BDC921D6C313740BA67D7760DC75571" ma:contentTypeVersion="9" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ec6cd274e87ab0abf30bec2e834aaf15">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="220d4249-f262-4642-a86b-ff46de6e315d" xmlns:ns3="965e701d-44ad-4371-a199-8fefe953808c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e77808c4f084d99d477d3de919e85b9" ns2:_="" ns3:_="">
     <xsd:import namespace="220d4249-f262-4642-a86b-ff46de6e315d"/>
@@ -2179,6 +2185,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC650EC1-3E41-4FC6-BA6C-52921951A8DA}">
   <ds:schemaRefs>
@@ -2191,14 +2206,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2190EF49-E186-4D77-87E3-BC317999ED9E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2215,4 +2222,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Web to resource sheet
</commit_message>
<xml_diff>
--- a/app/templates/report/recursos.xlsx
+++ b/app/templates/report/recursos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB8E3A73-690F-4BBF-A92D-4C5652B362CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08571B26-2BB2-4DAF-8CE4-CCF14C25ACD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Recursos" sheetId="37" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">_Precios!$A$2:$N$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BO$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Recursos!$A$2:$BP$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Valoraciones!$A$2:$F$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="162">
   <si>
     <t>Code</t>
   </si>
@@ -531,6 +531,12 @@
   </si>
   <si>
     <t>LAU_applicable</t>
+  </si>
+  <si>
+    <t>Web</t>
+  </si>
+  <si>
+    <t>Segment.Name</t>
   </si>
 </sst>
 </file>
@@ -1175,50 +1181,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BP3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BQ3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="37.28515625" style="2" customWidth="1"/>
-    <col min="3" max="4" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="20.42578125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="29.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.85546875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="20" width="12.28515625" style="2" customWidth="1"/>
-    <col min="21" max="28" width="9.5703125" style="2" customWidth="1"/>
-    <col min="29" max="29" width="53.7109375" style="2" customWidth="1"/>
-    <col min="30" max="30" width="10.7109375" style="2" customWidth="1"/>
-    <col min="31" max="31" width="30" style="2" customWidth="1"/>
-    <col min="32" max="32" width="24.7109375" style="2" customWidth="1"/>
-    <col min="33" max="33" width="11.85546875" style="31" customWidth="1"/>
-    <col min="34" max="35" width="11.5703125" style="2" customWidth="1"/>
-    <col min="36" max="37" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="10.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="11.5703125" style="2" customWidth="1"/>
-    <col min="40" max="40" width="10.7109375" style="2" customWidth="1"/>
-    <col min="41" max="41" width="14.140625" style="27" customWidth="1"/>
-    <col min="42" max="45" width="10.7109375" style="2" customWidth="1"/>
-    <col min="46" max="46" width="14.140625" style="27" customWidth="1"/>
-    <col min="47" max="51" width="11.85546875" style="2" customWidth="1"/>
-    <col min="52" max="54" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="55" max="56" width="15.42578125" style="2" customWidth="1"/>
-    <col min="57" max="58" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.7109375" style="2" customWidth="1"/>
-    <col min="61" max="62" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="63" max="66" width="16.85546875" style="2" customWidth="1"/>
-    <col min="67" max="67" width="20.5703125" style="2" customWidth="1"/>
-    <col min="68" max="68" width="5.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="69" max="16384" width="24.85546875" style="2"/>
+    <col min="1" max="2" width="37.33203125" style="2" customWidth="1"/>
+    <col min="3" max="4" width="20.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="20.44140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.88671875" style="2" customWidth="1"/>
+    <col min="13" max="13" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="12.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="21" width="12.33203125" style="2" customWidth="1"/>
+    <col min="22" max="29" width="9.5546875" style="2" customWidth="1"/>
+    <col min="30" max="30" width="53.6640625" style="2" customWidth="1"/>
+    <col min="31" max="31" width="10.6640625" style="2" customWidth="1"/>
+    <col min="32" max="32" width="30" style="2" customWidth="1"/>
+    <col min="33" max="33" width="24.6640625" style="2" customWidth="1"/>
+    <col min="34" max="34" width="11.88671875" style="31" customWidth="1"/>
+    <col min="35" max="36" width="11.5546875" style="2" customWidth="1"/>
+    <col min="37" max="38" width="17.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="10.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="11.5546875" style="2" customWidth="1"/>
+    <col min="41" max="41" width="10.6640625" style="2" customWidth="1"/>
+    <col min="42" max="42" width="14.109375" style="27" customWidth="1"/>
+    <col min="43" max="46" width="10.6640625" style="2" customWidth="1"/>
+    <col min="47" max="47" width="14.109375" style="27" customWidth="1"/>
+    <col min="48" max="52" width="11.88671875" style="2" customWidth="1"/>
+    <col min="53" max="55" width="17.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="56" max="57" width="15.44140625" style="2" customWidth="1"/>
+    <col min="58" max="59" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="12.6640625" style="2" customWidth="1"/>
+    <col min="62" max="63" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="64" max="67" width="16.88671875" style="2" customWidth="1"/>
+    <col min="68" max="68" width="20.5546875" style="2" customWidth="1"/>
+    <col min="69" max="69" width="5.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="70" max="16384" width="24.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:69" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1258,170 +1264,173 @@
         <v>8</v>
       </c>
       <c r="O1" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="AG1" s="28" t="s">
+      <c r="AH1" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="AH1" s="21" t="s">
+      <c r="AI1" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="AI1" s="21" t="s">
+      <c r="AJ1" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="AJ1" s="21" t="s">
+      <c r="AK1" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="AK1" s="21" t="s">
+      <c r="AL1" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="AL1" s="21" t="s">
+      <c r="AM1" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="AM1" s="21" t="s">
+      <c r="AN1" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="AN1" s="21" t="s">
+      <c r="AO1" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="AO1" s="21" t="s">
+      <c r="AP1" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="AP1" s="21" t="s">
+      <c r="AQ1" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="AQ1" s="21" t="s">
+      <c r="AR1" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="21" t="s">
+      <c r="AS1" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="AS1" s="21" t="s">
+      <c r="AT1" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="AT1" s="21" t="s">
+      <c r="AU1" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="AU1" s="32" t="s">
+      <c r="AV1" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="AV1" s="32" t="s">
+      <c r="AW1" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="AW1" s="32" t="s">
+      <c r="AX1" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="AX1" s="32" t="s">
+      <c r="AY1" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="AY1" s="3" t="s">
+      <c r="AZ1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="AZ1" s="3" t="s">
+      <c r="BA1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="BA1" s="3" t="s">
+      <c r="BB1" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BC1" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BD1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BE1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BF1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="BF1" s="3" t="s">
+      <c r="BG1" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="BG1" s="3" t="s">
+      <c r="BH1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="BH1" s="3" t="s">
+      <c r="BI1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="BI1" s="3" t="s">
+      <c r="BJ1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="BJ1" s="3" t="s">
+      <c r="BK1" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="BK1" s="3" t="s">
+      <c r="BL1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="BL1" s="3" t="s">
+      <c r="BM1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="BM1" s="3" t="s">
+      <c r="BN1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="BN1" s="3" t="s">
+      <c r="BO1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="BO1" s="3" t="s">
+      <c r="BP1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="BP1" s="1">
+      <c r="BQ1" s="1">
         <f ca="1">IF(MONTH(TODAY())&gt;8,1+YEAR(TODAY()),YEAR(TODAY()))</f>
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>67</v>
       </c>
@@ -1463,24 +1472,26 @@
         <v>3</v>
       </c>
       <c r="O2" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="P2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="R2" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="U2" s="4"/>
       <c r="V2" s="4"/>
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
@@ -1488,117 +1499,118 @@
       <c r="Z2" s="4"/>
       <c r="AA2" s="4"/>
       <c r="AB2" s="4"/>
-      <c r="AC2" s="4" t="s">
+      <c r="AC2" s="4"/>
+      <c r="AD2" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="AD2" s="4" t="s">
+      <c r="AE2" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="AE2" s="4" t="s">
+      <c r="AF2" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="AF2" s="4" t="s">
+      <c r="AG2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="AG2" s="29" t="s">
+      <c r="AH2" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="AH2" s="4" t="s">
+      <c r="AI2" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="AI2" s="4" t="s">
+      <c r="AJ2" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="AJ2" s="4" t="s">
+      <c r="AK2" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="AK2" s="4" t="s">
+      <c r="AL2" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="AL2" s="4" t="s">
+      <c r="AM2" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="AM2" s="4" t="s">
+      <c r="AN2" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="AN2" s="4" t="s">
+      <c r="AO2" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="AO2" s="25" t="s">
+      <c r="AP2" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="AP2" s="4" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AS2" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="AT2" s="25" t="s">
+      <c r="AU2" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="AU2" s="4"/>
       <c r="AV2" s="4"/>
       <c r="AW2" s="4"/>
       <c r="AX2" s="4"/>
-      <c r="AY2" s="4" t="s">
+      <c r="AY2" s="4"/>
+      <c r="AZ2" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="AZ2" s="4" t="s">
+      <c r="BA2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="BA2" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="BB2" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="BC2" s="4" t="s">
+      <c r="BD2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="BD2" s="4" t="s">
+      <c r="BE2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="BE2" s="4" t="s">
+      <c r="BF2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="BF2" s="4" t="s">
+      <c r="BG2" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="BG2" s="4" t="s">
+      <c r="BH2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="BH2" s="4" t="s">
+      <c r="BI2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="BI2" s="4" t="s">
+      <c r="BJ2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="BJ2" s="4" t="s">
+      <c r="BK2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="BK2" s="4" t="s">
+      <c r="BL2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="BL2" s="4" t="s">
+      <c r="BM2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="BM2" s="4" t="s">
+      <c r="BN2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="BN2" s="4" t="s">
+      <c r="BO2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="BO2" s="4" t="s">
+      <c r="BP2" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:69" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="10"/>
@@ -1619,70 +1631,70 @@
       <c r="R3" s="10"/>
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
-      <c r="U3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+      <c r="U3" s="10"/>
+      <c r="V3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
-      <c r="V3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+      <c r="W3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
-      <c r="W3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($O3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+      <c r="X3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
-      <c r="X3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
+      <c r="Y3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
         <v>0</v>
       </c>
-      <c r="Y3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BP$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
+      <c r="Z3" s="13">
+        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
         <v>0</v>
       </c>
-      <c r="Z3" s="13">
-        <f t="shared" ref="Z3" ca="1" si="0">$U3+$Y3</f>
+      <c r="AA3" s="13">
+        <f t="shared" ref="AA3" ca="1" si="0">$V3+$Z3</f>
         <v>0</v>
       </c>
-      <c r="AA3" s="13">
-        <f t="shared" ref="AA3" ca="1" si="1">$V3+$Y3</f>
+      <c r="AB3" s="13">
+        <f t="shared" ref="AB3" ca="1" si="1">$W3+$Z3</f>
         <v>0</v>
       </c>
-      <c r="AB3" s="13">
-        <f t="shared" ref="AB3" ca="1" si="2">$W3+$Y3</f>
+      <c r="AC3" s="13">
+        <f t="shared" ref="AC3" ca="1" si="2">$X3+$Z3</f>
         <v>0</v>
       </c>
-      <c r="AC3" s="20"/>
-      <c r="AD3" s="19" t="s">
+      <c r="AD3" s="20"/>
+      <c r="AE3" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="AE3" s="20"/>
-      <c r="AF3" s="17"/>
-      <c r="AG3" s="30"/>
-      <c r="AH3" s="22" t="s">
-        <v>96</v>
-      </c>
+      <c r="AF3" s="20"/>
+      <c r="AG3" s="17"/>
+      <c r="AH3" s="30"/>
       <c r="AI3" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="AJ3" s="24"/>
+      <c r="AJ3" s="22" t="s">
+        <v>96</v>
+      </c>
       <c r="AK3" s="24"/>
       <c r="AL3" s="24"/>
-      <c r="AM3" s="22" t="s">
+      <c r="AM3" s="24"/>
+      <c r="AN3" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="AN3" s="23"/>
-      <c r="AO3" s="26"/>
-      <c r="AP3" s="23"/>
+      <c r="AO3" s="23"/>
+      <c r="AP3" s="26"/>
       <c r="AQ3" s="23"/>
       <c r="AR3" s="23"/>
       <c r="AS3" s="23"/>
-      <c r="AT3" s="26"/>
-      <c r="AU3" s="33"/>
-      <c r="AV3" s="34"/>
+      <c r="AT3" s="23"/>
+      <c r="AU3" s="26"/>
+      <c r="AV3" s="33"/>
       <c r="AW3" s="34"/>
       <c r="AX3" s="34"/>
-      <c r="AY3" s="18"/>
-      <c r="AZ3" s="10"/>
+      <c r="AY3" s="34"/>
+      <c r="AZ3" s="18"/>
       <c r="BA3" s="10"/>
       <c r="BB3" s="10"/>
       <c r="BC3" s="10"/>
@@ -1698,10 +1710,11 @@
       <c r="BM3" s="10"/>
       <c r="BN3" s="10"/>
       <c r="BO3" s="10"/>
+      <c r="BP3" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BO3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A3:BO9988">
+  <autoFilter ref="A2:BP3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="A3:BP9988">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>LEN($D3)=12</formula>
     </cfRule>
@@ -1715,12 +1728,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E1D64B2-929E-46C9-92E4-4B6A6392A32E}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" style="2" customWidth="1"/>
     <col min="3" max="6" width="14" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="24.85546875" style="2"/>
+    <col min="7" max="16384" width="24.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1789,17 +1802,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F063E8C-9C12-4A86-8416-6A77642A363A}">
   <dimension ref="A1:S3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="24.85546875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.85546875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="40.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="18" width="17.7109375" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="24.85546875" style="2"/>
+    <col min="1" max="1" width="9.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="40.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="18" width="17.6640625" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="24.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1936,12 +1949,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F48469C1-5DA9-43F7-A0B7-76DC91FAD532}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="7.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ICal to resources report
</commit_message>
<xml_diff>
--- a/app/templates/report/recursos.xlsx
+++ b/app/templates/report/recursos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08571B26-2BB2-4DAF-8CE4-CCF14C25ACD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB8468D0-6EDA-46F9-874C-A22F71491367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="163">
   <si>
     <t>Code</t>
   </si>
@@ -537,6 +537,9 @@
   </si>
   <si>
     <t>Segment.Name</t>
+  </si>
+  <si>
+    <t>Ical</t>
   </si>
 </sst>
 </file>
@@ -1181,7 +1184,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BQ3"/>
+  <dimension ref="A1:BR3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="37.33203125" style="2" customWidth="1"/>
@@ -1220,11 +1223,12 @@
     <col min="62" max="63" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="64" max="67" width="16.88671875" style="2" customWidth="1"/>
     <col min="68" max="68" width="20.5546875" style="2" customWidth="1"/>
-    <col min="69" max="69" width="5.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="70" max="16384" width="24.88671875" style="2"/>
+    <col min="69" max="69" width="93.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="5.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="71" max="16384" width="24.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:70" s="1" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -1425,12 +1429,15 @@
       <c r="BP1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="BQ1" s="1">
+      <c r="BQ1" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="BR1" s="1">
         <f ca="1">IF(MONTH(TODAY())&gt;8,1+YEAR(TODAY()),YEAR(TODAY()))</f>
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>67</v>
       </c>
@@ -1609,8 +1616,9 @@
       <c r="BP2" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="BQ2" s="4"/>
     </row>
-    <row r="3" spans="1:69" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="10"/>
@@ -1633,23 +1641,23 @@
       <c r="T3" s="10"/>
       <c r="U3" s="10"/>
       <c r="V3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!H:H,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="W3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!I:I,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="X3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
+        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!J:J,0)*_xlfn.XLOOKUP($P3,_Tarifas!$A:$A,_Tarifas!C:C,0)*(1+0.01*_xlfn.NUMBERVALUE(SUBSTITUTE($L3,".",",")))</f>
         <v>0</v>
       </c>
       <c r="Y3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!K:K,0)</f>
         <v>0</v>
       </c>
       <c r="Z3" s="13">
-        <f ca="1">_xlfn.XLOOKUP($BQ$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
+        <f ca="1">_xlfn.XLOOKUP($BR$1&amp;LEFT($D3,6)&amp;$H3&amp;$J3,_Precios!$S:$S,_Precios!L:L,0)</f>
         <v>0</v>
       </c>
       <c r="AA3" s="13">
@@ -1711,10 +1719,11 @@
       <c r="BN3" s="10"/>
       <c r="BO3" s="10"/>
       <c r="BP3" s="10"/>
+      <c r="BQ3" s="10"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:BP3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="A3:BP9988">
+  <conditionalFormatting sqref="A3:BQ9988">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>LEN($D3)=12</formula>
     </cfRule>
@@ -2002,6 +2011,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001BDC921D6C313740BA67D7760DC75571" ma:contentTypeVersion="9" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ec6cd274e87ab0abf30bec2e834aaf15">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="220d4249-f262-4642-a86b-ff46de6e315d" xmlns:ns3="965e701d-44ad-4371-a199-8fefe953808c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e77808c4f084d99d477d3de919e85b9" ns2:_="" ns3:_="">
     <xsd:import namespace="220d4249-f262-4642-a86b-ff46de6e315d"/>
@@ -2198,15 +2216,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC650EC1-3E41-4FC6-BA6C-52921951A8DA}">
   <ds:schemaRefs>
@@ -2219,6 +2228,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2190EF49-E186-4D77-87E3-BC317999ED9E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2235,12 +2252,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91323775-37AE-44DC-8259-7FCDE5D849E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>